<commit_message>
Fixed Salary slip Interface
</commit_message>
<xml_diff>
--- a/backend/app/assets/payroll/AROMAZEN_Salary_Upload_Template.xlsx
+++ b/backend/app/assets/payroll/AROMAZEN_Salary_Upload_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary Data" sheetId="1" r:id="Rc6f7250307014bbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Ra4e8b1da40ac4b16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary Data" sheetId="1" r:id="R1e243f8d071c4961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R0e9544b6b6924666"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -126,12 +126,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">EMP001</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mangalore Unit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">B-105/106, Industrial Area, Baikampady, Mangalore - 575 011</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Executive</x:t>
@@ -1100,96 +1094,99 @@
       <x:c r="D2" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="E2" t="s">
+      <x:c r="E2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2"/>
+      <x:c r="G2" t="s">
         <x:v>39</x:v>
-      </x:c>
-      <x:c r="F2" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G2" t="s">
-        <x:v>41</x:v>
       </x:c>
       <x:c r="H2" s="2">
         <x:v>44571</x:v>
       </x:c>
       <x:c r="I2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="J2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="L2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="M2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="N2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="O2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="P2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="Q2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="R2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="S2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="T2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="U2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="V2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="W2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="X2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="Y2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="Z2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="AA2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="AB2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="AC2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="AD2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="AE2"/>
       <x:c r="AF2"/>
       <x:c r="AG2"/>
       <x:c r="AH2"/>
       <x:c r="AI2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="AJ2" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="E2:E502">
+      <x:formula1>"1,2,3"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -1208,12 +1205,12 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Use one row per employee. Employee name, personal email, date of birth, employee code, unit and unit address are mandatory.</x:v>
+        <x:v>Use one row per employee. Employee name, personal email, date of birth, employee code and Unit 1, 2 or 3 are mandatory. Unit Address can be left blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Enter the applicable unit and Unit Address. That address is printed on the employee's PDF.</x:v>
+        <x:v>The approved address is matched automatically from the Unit value and printed on that employee's salary slip.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1228,7 +1225,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>To change the design, export the approved Canva salary-slip page as a one-page A4 portrait PDF and upload it in Template Management.</x:v>
+        <x:v>One approved salary-slip master is used for every unit. Edit it in Canva, export one A4 portrait PDF and upload it in the Salary Slip Template Library.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>